<commit_message>
IEC general arrangement drawings GA-100..104 with installation and maintenance requirements
- temporary_codes/case_iec_documents/iec_drawings.py: A1 DXF + PDF drawings (power island
  arrangement, GT and generator, ST/generator/condenser, HRSG, GSUs) with withdrawal and
  maintenance spaces, laydown, crane coverage and pads, heavy-haul SPMT access and
  requirement tables; weights from DS-101..106 / REQ-001; automatic frame/overlap checks
- sources/iec: GA-100..104 Rev 0 registered (SRC-IECE-0009..0013)
- equipment records: positions and envelopes from the GAs (EPC load)
- plot_plan 1.1.0: linetype scale and text heights follow the drawing scale (site extents
  took minutes and were unreadable)
- TP-M1: heaviest piece corrected to the GT core engine 405 t; lesson L-EPCE-0003

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuQPCZMPzEzscTVqEEHFMo
</commit_message>
<xml_diff>
--- a/output/requirements_matrix/ALP_requirements_matrix.xlsx
+++ b/output/requirements_matrix/ALP_requirements_matrix.xlsx
@@ -493,7 +493,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T03:56:53Z by SETUP | data 5a092db99f236e4b</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T04:17:36Z by SETUP | data a69e0245c2d18fe7</t>
         </is>
       </c>
     </row>
@@ -8048,7 +8048,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T03:56:53Z by SETUP | data 5a092db99f236e4b</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T04:17:36Z by SETUP | data a69e0245c2d18fe7</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9295,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T03:56:53Z by SETUP | data 5a092db99f236e4b</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T04:17:36Z by SETUP | data a69e0245c2d18fe7</t>
         </is>
       </c>
     </row>
@@ -13081,7 +13081,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T03:56:53Z by SETUP | data 5a092db99f236e4b</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T04:17:36Z by SETUP | data a69e0245c2d18fe7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Proper document titles: '<Subject> - <Document Type>', explanations in a description column
- engine/core/titles.py: bracket split, title case (codes, units, acronyms kept), type/subject swap
- document / mdl_rule / gate_rule: new description field; rule titles '{name} - Type'; mdl sync
  maintains title and description; 2,061 rule documents and 177 single documents retitled, gates retitled
- MDL, release control (release plan, gates, gate rules) and procedure cover pages show the description
- fire water tanks A/B in one field-erected API 650 package (MR-ME-017) with one datasheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuQPCZMPzEzscTVqEEHFMo
</commit_message>
<xml_diff>
--- a/output/requirements_matrix/ALP_requirements_matrix.xlsx
+++ b/output/requirements_matrix/ALP_requirements_matrix.xlsx
@@ -485,7 +485,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T17:23:32Z by SETUP | data 9c5db87d3bb3d7c9</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T18:43:04Z by SETUP | data 320a8d5c2b38b7e8</t>
         </is>
       </c>
     </row>
@@ -646,6 +646,7 @@
       <c r="J6" s="5" t="inlineStr">
         <is>
           <t>document/ALP-EPC-00000-GE-DBR-0001
+document/ALP-EPC-00000-PR-DBR-0001
 document/ALP-EPC-00000-PR-PFD-0002
 document/ALP-EPC-00EGA-ME-CAL-0001
 document/ALP-EPC-00EGA-PI-ISO-0001
@@ -859,6 +860,8 @@
 document/ALP-EPC-20MAN-PR-SDS-0001
 document/ALP-EPC-20UMB-PI-LAY-0001
 document/ALP-EPC-20UMB-PI-PPL-0001
+mdl_rule/DL-DBR-GE
+mdl_rule/DL-DBR-PR
 mdl_rule/DL-ME-CAL
 mdl_rule/DL-PI-ISO
 mdl_rule/DL-PI-LAY
@@ -1569,7 +1572,9 @@
           <t>design_parameter/DP-CASE-0001
 design_parameter/DP-OWNR-0044
 document/ALP-EPC-00000-CV-RPT-0003
-document/ALP-EPC-00000-GE-DBR-0001</t>
+document/ALP-EPC-00000-GE-DBR-0001
+document/ALP-EPC-00000-PR-DBR-0001
+mdl_rule/DL-DBR-PR</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -1947,8 +1952,10 @@
         <is>
           <t>design_parameter/DP-CASE-0003
 document/ALP-EPC-00000-EL-CAL-0005
+document/ALP-EPC-00000-ME-DBR-0001
 document/ALP-EPC-00000-ME-RPT-0002
 document/ALP-EPC-00000-ME-SPC-0002
+mdl_rule/DL-DBR-ME
 mr/MR-EL-010
 mr/MR-ME-022</t>
         </is>
@@ -5627,7 +5634,8 @@
       <c r="I91" s="4" t="inlineStr"/>
       <c r="J91" s="5" t="inlineStr">
         <is>
-          <t>document/ALP-EPC-00EGA-ME-DSH-0001
+          <t>document/ALP-EPC-00000-ME-DBR-0001
+document/ALP-EPC-00EGA-ME-DSH-0001
 document/ALP-EPC-00EGA-ME-DSH-0002
 document/ALP-EPC-00EGA-ME-DSH-0003
 document/ALP-EPC-00EGA-ME-DSH-0004
@@ -5715,6 +5723,7 @@
 document/ALP-EPC-10LAC-ME-DSH-0001
 document/ALP-EPC-10LAC-PR-SDS-0001
 document/ALP-EPC-20LCB-ME-DSH-0001
+mdl_rule/DL-DBR-ME
 mdl_rule/DL-ME-DSH
 mr/MR-PI-006</t>
         </is>
@@ -6011,7 +6020,8 @@
       <c r="I96" s="4" t="inlineStr"/>
       <c r="J96" s="5" t="inlineStr">
         <is>
-          <t>document/ALP-EPC-00SAA-HV-SDS-0001
+          <t>document/ALP-EPC-00000-HV-DBR-0001
+document/ALP-EPC-00SAA-HV-SDS-0001
 document/ALP-EPC-00UAC-HV-GAD-0001
 document/ALP-EPC-00UBA-HV-GAD-0001
 document/ALP-EPC-00UBA-HV-GAD-0002
@@ -6026,6 +6036,7 @@
 document/ALP-EPC-10UMA-HV-GAD-0001
 document/ALP-EPC-10UMA-HV-GAD-0002
 document/ALP-EPC-20UMB-HV-GAD-0001
+mdl_rule/DL-DBR-HV
 mdl_rule/DL-HV-HVL
 mdl_rule/DL-HV-SRV</t>
         </is>
@@ -6330,7 +6341,8 @@
       <c r="I102" s="4" t="inlineStr"/>
       <c r="J102" s="5" t="inlineStr">
         <is>
-          <t>document/ALP-EPC-00000-EL-RPT-0001
+          <t>document/ALP-EPC-00000-EL-DBR-0001
+document/ALP-EPC-00000-EL-RPT-0001
 document/ALP-EPC-00ACA-EL-DSH-0001
 document/ALP-EPC-00BBA-EL-DSH-0001
 document/ALP-EPC-00BBA-EL-SLD-0001
@@ -6357,6 +6369,7 @@
 document/ALP-EPC-00XJA-EL-DSH-0001
 document/ALP-EPC-10BBT-EL-DSH-0001
 document/ALP-EPC-20BBT-EL-DSH-0001
+mdl_rule/DL-DBR-EL
 mdl_rule/DL-EL-DSH
 mdl_rule/DL-EL-WLV
 mdl_rule/DL-EL-WMV</t>
@@ -6728,7 +6741,8 @@
       <c r="I108" s="4" t="inlineStr"/>
       <c r="J108" s="5" t="inlineStr">
         <is>
-          <t>document/ALP-EPC-00000-IC-SPC-0005
+          <t>document/ALP-EPC-00000-IC-DBR-0001
+document/ALP-EPC-00000-IC-SPC-0005
 document/ALP-EPC-00000-IC-TST-0001
 document/ALP-EPC-00ACA-IC-DSH-0001
 document/ALP-EPC-00CJA-IC-BLK-0001
@@ -6862,6 +6876,7 @@
 document/ALP-EPC-20UMB-IC-HUP-0001
 document/ALP-EPC-20UMB-IC-LOP-0001
 document/ALP-EPC-20UMB-IC-LOP-0002
+mdl_rule/DL-DBR-IC
 mdl_rule/DL-IC-BLK
 mdl_rule/DL-IC-DSH
 mdl_rule/DL-IC-HUP
@@ -7478,6 +7493,7 @@
       <c r="J116" s="5" t="inlineStr">
         <is>
           <t>document/ALP-EPC-00000-CV-CAL-0001
+document/ALP-EPC-00000-CV-DBR-0001
 document/ALP-EPC-00000-CV-TRP-0001
 document/ALP-EPC-00000-CV-TST-0001
 document/ALP-EPC-00UAC-CV-CAL-0001
@@ -7542,7 +7558,8 @@
 mdl_rule/DL-CV-CAL
 mdl_rule/DL-CV-EFD
 mdl_rule/DL-CV-FND
-mdl_rule/DL-CV-PIL</t>
+mdl_rule/DL-CV-PIL
+mdl_rule/DL-DBR-CV</t>
         </is>
       </c>
       <c r="K116" s="4" t="inlineStr">
@@ -8110,7 +8127,9 @@
       <c r="J124" s="5" t="inlineStr">
         <is>
           <t>design_parameter/DP-CASE-0044
-document/ALP-EPC-00000-HS-STU-0001</t>
+document/ALP-EPC-00000-HS-DBR-0001
+document/ALP-EPC-00000-HS-STU-0001
+mdl_rule/DL-DBR-HS</t>
         </is>
       </c>
       <c r="K124" s="4" t="inlineStr">
@@ -8247,6 +8266,7 @@
 document/ALP-E12-00000-GE-MOS-0004
 document/ALP-E12-00000-GE-MOS-0005
 document/ALP-E12-00000-GE-MOS-0006
+document/ALP-EPC-00000-HS-DBR-0001
 document/ALP-EPC-00000-HS-PLN-0001
 document/ALP-EPC-00000-HS-PLN-0002
 document/ALP-EPC-00000-HS-PLN-0005
@@ -8287,6 +8307,7 @@
 document/ALP-S02-10HNE-GE-MOS-0004
 document/ALP-S02-10HNE-GE-MOS-0005
 document/ALP-S02-10HNE-GE-MOS-0006
+mdl_rule/DL-DBR-HS
 mdl_rule/DL-S-MOS
 permit/PMT-010</t>
         </is>
@@ -8394,10 +8415,12 @@
       <c r="I128" s="4" t="inlineStr"/>
       <c r="J128" s="5" t="inlineStr">
         <is>
-          <t>document/ALP-EPC-00000-HS-HAZ-0002
+          <t>document/ALP-EPC-00000-HS-DBR-0001
+document/ALP-EPC-00000-HS-HAZ-0002
 document/ALP-EPC-00000-HS-HAZ-0010
 document/ALP-EPC-00000-HS-RPT-0004
-document/ALP-EPC-00000-PR-RPT-0003</t>
+document/ALP-EPC-00000-PR-RPT-0003
+mdl_rule/DL-DBR-HS</t>
         </is>
       </c>
       <c r="K128" s="4" t="inlineStr">
@@ -8773,6 +8796,9 @@
 document/ALP-M24-00UZF-GE-ITP-0001
 document/ALP-S01-00000-GE-ITP-0001
 document/ALP-S02-10HNE-GE-ITP-0001
+gate_rule/G-PRC-ENQ
+gate_rule/G-PRC-FAB
+gate_rule/G-PRC-PO
 mdl_rule/DL-MR-ITP
 mdl_rule/DL-MR-MRQ
 mdl_rule/DL-MR-SPC
@@ -8914,6 +8940,8 @@
 document/ALP-M20-00SGA-ME-TST-0001
 document/ALP-M21-00SMA-ME-TRP-0001
 document/ALP-M21-00SMA-ME-TST-0001
+gate_rule/G-PRC-FAT
+gate_rule/G-PRC-SHP
 mdl_rule/DL-V-FAT
 mdl_rule/DL-V-FTR</t>
         </is>
@@ -9045,6 +9073,7 @@
 document/ALP-P05-00000-ME-MDB-0001
 document/ALP-P06-00000-ME-MDB-0001
 document/ALP-P07-00000-ME-MDB-0001
+gate_rule/G-PRC-SHP
 mdl_rule/DL-PR-PSV
 mdl_rule/DL-V-MDB
 mr/MR-PI-007</t>
@@ -9200,6 +9229,7 @@
 document/ALP-EPC-00GMA-CM-MDB-0001
 document/ALP-EPC-00GNA-CM-CMP-0001
 document/ALP-EPC-00GNA-CM-MDB-0001
+document/ALP-EPC-00GQA-CM-MDB-0001
 document/ALP-EPC-00GUA-CM-CMP-0001
 document/ALP-EPC-00GUA-CM-MDB-0001
 document/ALP-EPC-00LBG-CM-CMP-0001
@@ -9242,12 +9272,18 @@
 document/ALP-EPC-00SMA-CM-MDB-0001
 document/ALP-EPC-00XJA-CM-CMP-0001
 document/ALP-EPC-00XJA-CM-MDB-0001
+document/ALP-EPC-10BAA-CM-MDB-0001
+document/ALP-EPC-10BAC-CM-MDB-0001
+document/ALP-EPC-10BAT-CM-MDB-0001
 document/ALP-EPC-10BBT-CM-CMP-0001
 document/ALP-EPC-10BBT-CM-MDB-0001
+document/ALP-EPC-10HAA-CM-MDB-0001
 document/ALP-EPC-10HAN-CM-CMP-0001
 document/ALP-EPC-10HAN-CM-MDB-0001
+document/ALP-EPC-10HNA-CM-MDB-0001
 document/ALP-EPC-10HNE-CM-CMP-0001
 document/ALP-EPC-10HNE-CM-MDB-0001
+document/ALP-EPC-10HSA-CM-MDB-0001
 document/ALP-EPC-10HSB-CM-CMP-0001
 document/ALP-EPC-10HSB-CM-MDB-0001
 document/ALP-EPC-10LAB-CM-CMP-0001
@@ -9266,20 +9302,49 @@
 document/ALP-EPC-10LBC-CM-MDB-0001
 document/ALP-EPC-10LBD-CM-CMP-0001
 document/ALP-EPC-10LBD-CM-MDB-0001
+document/ALP-EPC-10MBA-CM-MDB-0001
+document/ALP-EPC-10MBL-CM-MDB-0001
+document/ALP-EPC-10MBN-CM-MDB-0001
+document/ALP-EPC-10MBP-CM-MDB-0001
+document/ALP-EPC-10MBU-CM-MDB-0001
+document/ALP-EPC-10MBV-CM-MDB-0001
+document/ALP-EPC-10MBY-CM-MDB-0001
+document/ALP-EPC-10MKA-CM-MDB-0001
+document/ALP-EPC-10MKC-CM-MDB-0001
+document/ALP-EPC-10MKG-CM-MDB-0001
+document/ALP-EPC-20BAA-CM-MDB-0001
+document/ALP-EPC-20BAC-CM-MDB-0001
+document/ALP-EPC-20BAT-CM-MDB-0001
 document/ALP-EPC-20BBT-CM-CMP-0001
 document/ALP-EPC-20BBT-CM-MDB-0001
 document/ALP-EPC-20LCA-CM-CMP-0001
 document/ALP-EPC-20LCA-CM-MDB-0001
 document/ALP-EPC-20LCB-CM-CMP-0001
 document/ALP-EPC-20LCB-CM-MDB-0001
+document/ALP-EPC-20MAA-CM-MDB-0001
+document/ALP-EPC-20MAB-CM-MDB-0001
+document/ALP-EPC-20MAG-CM-MDB-0001
+document/ALP-EPC-20MAJ-CM-MDB-0001
 document/ALP-EPC-20MAN-CM-CMP-0001
 document/ALP-EPC-20MAN-CM-MDB-0001
+document/ALP-EPC-20MAV-CM-MDB-0001
+document/ALP-EPC-20MAW-CM-MDB-0001
+document/ALP-EPC-20MAX-CM-MDB-0001
+document/ALP-EPC-20MAY-CM-MDB-0001
+document/ALP-EPC-20MKA-CM-MDB-0001
+document/ALP-EPC-20MKC-CM-MDB-0001
 document/ALP-IEC-10BAT-CM-CMP-0001
 document/ALP-IEC-10HAA-CM-CMP-0001
 document/ALP-IEC-10MBA-CM-CMP-0001
 document/ALP-IEC-10MBY-CM-CMP-0001
 document/ALP-IEC-10MKA-CM-CMP-0001
 document/ALP-IEC-20MAA-CM-CMP-0001
+gate_rule/G-COM-MC-EL
+gate_rule/G-COM-MC-FF
+gate_rule/G-COM-MC-WS
+gate_rule/G-COM-SC-EL
+gate_rule/G-COM-SC-FF
+gate_rule/G-COM-SC-WS
 mdl_rule/DL-CM-CMP
 mdl_rule/DL-CM-TOD
 mdl_rule/DL-V-CMP</t>
@@ -9452,7 +9517,8 @@
       <c r="J138" s="5" t="inlineStr">
         <is>
           <t>document/ALP-EPC-00000-CM-CMP-0002
-document/ALP-EPC-00000-CM-TRP-0002</t>
+document/ALP-EPC-00000-CM-TRP-0002
+gate_rule/G-OWN-TOC</t>
         </is>
       </c>
       <c r="K138" s="4" t="inlineStr">
@@ -9747,7 +9813,8 @@
       <c r="I143" s="4" t="inlineStr"/>
       <c r="J143" s="5" t="inlineStr">
         <is>
-          <t>document/ALP-EPC-00000-GE-PRC-0002</t>
+          <t>document/ALP-EPC-00000-GE-PRC-0002
+gate_rule/G-OWN-BDP</t>
         </is>
       </c>
       <c r="K143" s="4" t="inlineStr">
@@ -9849,7 +9916,8 @@
         <is>
           <t>document/ALP-EPC-00000-GE-LST-0005
 document/ALP-EPC-00000-GE-PRC-0003
-document/ALP-EPC-00000-PI-M3D-0004</t>
+document/ALP-EPC-00000-PI-M3D-0004
+gate_rule/G-OPS-AB</t>
         </is>
       </c>
       <c r="K145" s="4" t="inlineStr">
@@ -10002,6 +10070,12 @@
 document/ALP-M19-10HAN-ME-OMM-0001
 document/ALP-M20-00SGA-ME-OMM-0001
 document/ALP-M21-00SMA-ME-OMM-0001
+gate_rule/G-COM-SC-EL
+gate_rule/G-COM-SC-FF
+gate_rule/G-COM-SC-WS
+gate_rule/G-OPS-HO-EL
+gate_rule/G-OPS-HO-FF
+gate_rule/G-OPS-HO-WS
 mdl_rule/DL-CM-OPR
 mdl_rule/DL-V-OMM</t>
         </is>
@@ -10149,6 +10223,7 @@
 document/ALP-M19-10HAN-ME-LST-0001
 document/ALP-M20-00SGA-ME-LST-0001
 document/ALP-M21-00SMA-ME-LST-0001
+gate_rule/G-OWN-TO
 mdl_rule/DL-V-SPL</t>
         </is>
       </c>
@@ -10504,7 +10579,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T17:23:32Z by SETUP | data 9c5db87d3bb3d7c9</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T18:43:04Z by SETUP | data 320a8d5c2b38b7e8</t>
         </is>
       </c>
     </row>
@@ -11751,7 +11826,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T17:23:32Z by SETUP | data 9c5db87d3bb3d7c9</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T18:43:04Z by SETUP | data 320a8d5c2b38b7e8</t>
         </is>
       </c>
     </row>
@@ -15537,7 +15612,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T17:23:32Z by SETUP | data 9c5db87d3bb3d7c9</t>
+          <t>engine requirements_matrix v1.0.0 | generated 2026-09-28T18:43:04Z by SETUP | data 320a8d5c2b38b7e8</t>
         </is>
       </c>
     </row>

</xml_diff>